<commit_message>
Update backend application structure and database files
- Modify models, schemas, and main application files
- Update database and Excel table files
- Remove old backend data.db file

🤖 Generated with [Claude Code](https://claude.ai/code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/db/tabla_unique_16.xlsx
+++ b/db/tabla_unique_16.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benjaminserranobarba/Desktop/Trabajo/web-app/db/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benjaminserranobarba/Desktop/Trabajo/web-app/estadia-back/db/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6299B804-E4D9-A041-BD78-9CE7AE3C5413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1380AD70-8093-BC4A-87B1-584EF57E3087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>